<commit_message>
A2: comps corrigés — faits, dé-hardcoding des fourchettes, bannière de péremption
Transaction_comps: Billtrust->EQT (2022), Bottomline->Thoma Bravo, Esker
EV 1091->1576 M / CA 158->205,3 M (7,7x CA 2024A), EBITDA Esker exclu des
agrégats (n.d.). Fourchette sélectionnée = formules sur les EV implicites
(289/411/547, quasi inchangée — midpoint 6,7x validé par le doc d'offre).

Trading_comps: ligne Esker restatée, bannière STALE datée (multiples H1-2025
à rafraîchir, métriques non homogènes), fourchette sélectionnée = moyenne
des méthodes Sales/EBITDA (211/361/548 vs 185/295/425 saisi en dur).
La 'convergence' construite trading 295 = DCF 301 disparaît: le football
field montre désormais un écart honnête DCF 301 vs trading 361.
Vérification: zéro erreur de formule, football field 100% dynamique.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Sidetrade_Valuation_2026_v2.xlsx
+++ b/Sidetrade_Valuation_2026_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Abbah\Downloads\Portefolio\Portefolio\Sidetrade\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90046EA8-93B2-4ADE-91CA-FC1F0520E702}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEABC4CA-E2F6-48EC-A88B-F64CDC90A3C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21840" tabRatio="500" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="922" uniqueCount="732">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="924" uniqueCount="732">
   <si>
     <t>LBO AFFORDABILITY MODEL — BASE CASE  |  Max Entry EV for IRR targets</t>
   </si>
@@ -1085,7 +1085,7 @@
     <t>TRADING COMPS — SaaS B2B / Finance Automation / O2C peers  |  Forward multiples FY2026E</t>
   </si>
   <si>
-    <t>EUR-translated at ~1.10 USD/EUR. Multiples approx. H1-2025. Update if market moves materially.</t>
+    <t>ATTENTION - Multiples approx. H1-2025, PERIMES: rafraichir prix/guidances 2026 des 4 peers avant toute diffusion (sources: communiques guidance 2026, cf. note audit 12.5). Metriques non homogenes entre peers (EBITDA adj. / non-GAAP OI). EUR/USD ~1.10. Derniere revue: 15-Jul-2026.</t>
   </si>
   <si>
     <t>Company</t>
@@ -1172,7 +1172,10 @@
     <t>O2C SaaS — Bridgepoint/GA acq. 2024</t>
   </si>
   <si>
-    <t>* Last traded pre-announcement. Deal: 6.9× FY25E Sales, 34.6× EBITDA</t>
+    <t>"n.m."</t>
+  </si>
+  <si>
+    <t>* Last traded pre-announcement. Deal 2024: ~7,7x CA 2024A / ~6,9x FY25E Sales (doc offre). EBITDA n.d.</t>
   </si>
   <si>
     <t>AGGREGATES (excl. Esker * reference row — row 9)</t>
@@ -1223,7 +1226,7 @@
     <t>Selected trading comp range  (€m EV)</t>
   </si>
   <si>
-    <t>Consistent with Valo.docx synthesis. Midpoint aligns with DCF Base.</t>
+    <t>Derive: moyenne des EV implicites Sales/EBITDA aux multiples retenus (l.21/23). Plus de midpoint saisi en dur (audit 4.4) - la fourchette bouge si les multiples ou le DCF bougent.</t>
   </si>
   <si>
     <t>* Esker (row 9): taken private. Included as directional reference only; use Transaction_comps for control multiples.</t>
@@ -1232,7 +1235,7 @@
     <t>TRANSACTION COMPS — Precedent M&amp;A in Office-of-CFO / O2C / Fintech SaaS  (control transactions)</t>
   </si>
   <si>
-    <t>All deals include control premium (30-50% vs. trading). Not directly comparable to stand-alone DCF/trading EV.</t>
+    <t>All deals include control premium (30-50% vs. trading). Faits verifies et corriges le 15-Jul-2026 (audit 4.5): Billtrust-&gt;EQT, Bottomline-&gt;Thoma Bravo, Esker EV/CA restates.</t>
   </si>
   <si>
     <t>Target</t>
@@ -1268,7 +1271,7 @@
     <t>O2C / AR automation (France)</t>
   </si>
   <si>
-    <t>Best read-across: same vertical, Euronext Growth, enterprise O2C</t>
+    <t>Offre 262 EUR/action (sept. 2024): equity ~1 619 M, EV ~1 576 M; ~7,7x CA 2024A (205,3 M). Doc offre: moyenne transactions ~6,8x NTM Sales. EBITDA LTM non retraite -&gt; exclu des agregats.</t>
   </si>
   <si>
     <t>Coupa</t>
@@ -1286,13 +1289,13 @@
     <t>Billtrust</t>
   </si>
   <si>
-    <t>Corpay (FLYW)</t>
+    <t>EQT Private Equity</t>
   </si>
   <si>
     <t>AR invoicing / cash app SaaS</t>
   </si>
   <si>
-    <t>~$1.75B; ~9× Sales; scale player AR automation</t>
+    <t>~USD 1,7 Md take-private (annonce sept. 2022); ~9x Sales; scale player AR automation</t>
   </si>
   <si>
     <t>Pagero</t>
@@ -1310,9 +1313,6 @@
     <t>Bottomline Tech.</t>
   </si>
   <si>
-    <t>Symphony Technology</t>
-  </si>
-  <si>
     <t>B2B payments / cash management</t>
   </si>
   <si>
@@ -1322,7 +1322,7 @@
     <t>AGGREGATES</t>
   </si>
   <si>
-    <t>Coupa excluded from EBITDA aggregates (near-breakeven at deal, 161.6x n/m)</t>
+    <t>Coupa (161x n/m) et Esker (EBITDA n.d.) exclus des agregats EV/EBITDA</t>
   </si>
   <si>
     <t>IMPLIED CONTROL EV FOR SIDETRADE</t>
@@ -1358,7 +1358,7 @@
     <t>Selected transaction comp range  (€m EV)</t>
   </si>
   <si>
-    <t>Control premium ~40% vs. stand-alone. Base €410m consistent with Valo.docx.</t>
+    <t>Derive des multiples ligne 24 (mid = moyenne doc offre Esker ~6,8x NTM avec decote taille). Control premium ~40% vs stand-alone.</t>
   </si>
   <si>
     <t>IMPORTANT: Transaction comps include control premium. NOT directly comparable to DCF or trading comp EV.</t>
@@ -3298,7 +3298,7 @@
       </c>
       <c r="B12" s="13">
         <f>Transaction_comps!F27</f>
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="C12" s="14" t="s">
         <v>57</v>
@@ -3353,15 +3353,15 @@
       </c>
       <c r="B17" s="23">
         <f>Trading_comps!E26</f>
-        <v>185</v>
+        <v>211</v>
       </c>
       <c r="C17" s="23">
         <f>Trading_comps!F26</f>
-        <v>295</v>
+        <v>361</v>
       </c>
       <c r="D17" s="23">
         <f>Trading_comps!G26</f>
-        <v>425</v>
+        <v>548</v>
       </c>
       <c r="E17" s="24" t="s">
         <v>66</v>
@@ -3373,15 +3373,15 @@
       </c>
       <c r="B18" s="20">
         <f>Transaction_comps!E27</f>
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C18" s="20">
         <f>Transaction_comps!F27</f>
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="D18" s="20">
         <f>Transaction_comps!G27</f>
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="E18" s="21" t="s">
         <v>68</v>
@@ -7576,23 +7576,23 @@
       </c>
       <c r="B6" s="89">
         <f>Trading_comps!E26</f>
-        <v>185</v>
+        <v>211</v>
       </c>
       <c r="C6" s="89">
         <f>Trading_comps!F26</f>
-        <v>295</v>
+        <v>361</v>
       </c>
       <c r="D6" s="89">
         <f>Trading_comps!G26</f>
-        <v>425</v>
+        <v>548</v>
       </c>
       <c r="E6" s="90">
         <f>C6/Inputs!B7</f>
-        <v>22.041243275552898</v>
+        <v>26.972504482964734</v>
       </c>
       <c r="F6" s="90">
         <f>C6/Inputs!B6</f>
-        <v>4.8033085840823242</v>
+        <v>5.8779471147583697</v>
       </c>
       <c r="G6" s="91" t="s">
         <v>653</v>
@@ -7604,23 +7604,23 @@
       </c>
       <c r="B7" s="92">
         <f>Transaction_comps!E27</f>
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C7" s="92">
         <f>Transaction_comps!F27</f>
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="D7" s="92">
         <f>Transaction_comps!G27</f>
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="E7" s="93">
         <f>C7/Inputs!B7</f>
-        <v>30.63359234907352</v>
+        <v>30.708308427973698</v>
       </c>
       <c r="F7" s="93">
         <f>C7/Inputs!B6</f>
-        <v>6.6757848117754337</v>
+        <v>6.6920672137553732</v>
       </c>
       <c r="G7" s="94" t="s">
         <v>655</v>
@@ -7689,7 +7689,7 @@
       </c>
       <c r="C12" s="98">
         <f>Transaction_comps!F27</f>
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -7705,7 +7705,7 @@
       </c>
       <c r="D13" s="72">
         <f>Trading_comps!G26</f>
-        <v>425</v>
+        <v>548</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -7732,11 +7732,11 @@
       </c>
       <c r="B17" s="101" t="str">
         <f>REPT("░",ROUND(B6/600*48,0))&amp;REPT("█",MAX(1,ROUND((D6-B6)/600*48,0)))&amp;REPT("░",MAX(0,48-ROUND(B6/600*48,0)-MAX(1,ROUND((D6-B6)/600*48,0))))</f>
-        <v>░░░░░░░░░░░░░░░███████████████████░░░░░░░░░░░░░░</v>
+        <v>░░░░░░░░░░░░░░░░░███████████████████████████░░░░</v>
       </c>
       <c r="C17" s="102" t="str">
         <f>"Low €"&amp;TEXT(B6,"0")&amp;"m  |  Base €"&amp;TEXT(C6,"0")&amp;"m  |  High €"&amp;TEXT(D6,"0")&amp;"m"</f>
-        <v>Low €185m  |  Base €295m  |  High €425m</v>
+        <v>Low €211m  |  Base €361m  |  High €548m</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -7745,11 +7745,11 @@
       </c>
       <c r="B18" s="101" t="str">
         <f>REPT("░",ROUND(B7/600*48,0))&amp;REPT("█",MAX(1,ROUND((D7-B7)/600*48,0)))&amp;REPT("░",MAX(0,48-ROUND(B7/600*48,0)-MAX(1,ROUND((D7-B7)/600*48,0))))</f>
-        <v>░░░░░░░░░░░░░░░░░░░░░░░████████████████████░░░░░</v>
+        <v>░░░░░░░░░░░░░░░░░░░░░░░█████████████████████░░░░</v>
       </c>
       <c r="C18" s="102" t="str">
         <f>"Low €"&amp;TEXT(B7,"0")&amp;"m  |  Base €"&amp;TEXT(C7,"0")&amp;"m  |  High €"&amp;TEXT(D7,"0")&amp;"m"</f>
-        <v>Low €290m  |  Base €410m  |  High €545m</v>
+        <v>Low €289m  |  Base €411m  |  High €547m</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
@@ -8032,7 +8032,7 @@
       </c>
       <c r="C23" s="52">
         <f>Transaction_comps!F27</f>
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
@@ -8041,7 +8041,7 @@
       </c>
       <c r="C24" s="51">
         <f>C23-C12</f>
-        <v>395.346</v>
+        <v>396.346</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -8050,7 +8050,7 @@
       </c>
       <c r="C25" s="107">
         <f>C24/C19</f>
-        <v>257.2544069131111</v>
+        <v>257.90511390625915</v>
       </c>
       <c r="E25" s="28" t="s">
         <v>688</v>
@@ -12093,29 +12093,26 @@
         <v>374</v>
       </c>
       <c r="D9" s="66">
-        <v>1091</v>
+        <v>1576</v>
       </c>
       <c r="E9" s="66">
-        <v>158</v>
-      </c>
-      <c r="F9" s="66">
-        <v>32</v>
-      </c>
+        <v>205.3</v>
+      </c>
+      <c r="F9" s="66"/>
       <c r="G9" s="67">
         <f>D9/E9</f>
-        <v>6.9050632911392409</v>
-      </c>
-      <c r="H9" s="67">
-        <f>D9/F9</f>
-        <v>34.09375</v>
+        <v>7.6765708718947874</v>
+      </c>
+      <c r="H9" s="67" t="s">
+        <v>375</v>
       </c>
       <c r="I9" s="68" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="156" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="B11" s="146"/>
       <c r="C11" s="146"/>
@@ -12128,7 +12125,7 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="G12" s="42">
         <f>MEDIAN(G5:G8)</f>
@@ -12141,7 +12138,7 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="G13" s="42">
         <f>MIN(G5:G8)</f>
@@ -12154,7 +12151,7 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="G14" s="42">
         <f>MAX(G5:G8)</f>
@@ -12167,7 +12164,7 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="156" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="B16" s="146"/>
       <c r="C16" s="146"/>
@@ -12180,7 +12177,7 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="E17" s="72">
         <f>DCF!C7</f>
@@ -12189,7 +12186,7 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="9" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="F18" s="72">
         <f>DCF!C12</f>
@@ -12198,21 +12195,21 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="7" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="E20" s="18" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="F20" s="18" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="G20" s="18" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="9" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="E21" s="41">
         <v>3</v>
@@ -12226,7 +12223,7 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="E22" s="51">
         <f>E17*E21</f>
@@ -12243,7 +12240,7 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="9" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="E23" s="41">
         <v>12</v>
@@ -12257,7 +12254,7 @@
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="9" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="E24" s="51">
         <f>F18*E23</f>
@@ -12274,24 +12271,27 @@
     </row>
     <row r="26" spans="1:9" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="7" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="E26" s="52">
-        <v>185</v>
+        <f>ROUND(AVERAGE(E22,E24),0)</f>
+        <v>211</v>
       </c>
       <c r="F26" s="52">
-        <v>295</v>
+        <f>ROUND(AVERAGE(F22,F24),0)</f>
+        <v>361</v>
       </c>
       <c r="G26" s="52">
-        <v>425</v>
+        <f>ROUND(AVERAGE(G22,G24),0)</f>
+        <v>548</v>
       </c>
       <c r="I26" s="28" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="14" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
     </row>
   </sheetData>
@@ -12320,7 +12320,7 @@
   <sheetData>
     <row r="1" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="147" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="B1" s="146"/>
       <c r="C1" s="146"/>
@@ -12334,36 +12334,36 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="73" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>350</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>28</v>
@@ -12371,50 +12371,47 @@
     </row>
     <row r="5" spans="1:10" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="71" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="B5" s="74">
         <v>2024</v>
       </c>
       <c r="C5" s="65" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="D5" s="65" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="E5" s="66">
-        <v>1091</v>
+        <v>1576</v>
       </c>
       <c r="F5" s="66">
-        <v>158</v>
-      </c>
-      <c r="G5" s="66">
-        <v>32</v>
-      </c>
+        <v>205.3</v>
+      </c>
+      <c r="G5" s="66"/>
       <c r="H5" s="67">
         <f>E5/F5</f>
-        <v>6.9050632911392409</v>
-      </c>
-      <c r="I5" s="67">
-        <f>E5/G5</f>
-        <v>34.09375</v>
+        <v>7.6765708718947874</v>
+      </c>
+      <c r="I5" s="67" t="s">
+        <v>375</v>
       </c>
       <c r="J5" s="68" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="22" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="B6" s="75">
         <v>2023</v>
       </c>
       <c r="C6" s="29" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="D6" s="29" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="E6" s="69">
         <v>7273</v>
@@ -12434,21 +12431,21 @@
         <v>161.62222222222223</v>
       </c>
       <c r="J6" s="24" t="s">
-        <v>411</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A7" s="71" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="B7" s="74">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C7" s="65" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="D7" s="65" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="E7" s="66">
         <v>1591</v>
@@ -12468,21 +12465,21 @@
         <v>79.55</v>
       </c>
       <c r="J7" s="68" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="22" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="B8" s="75">
         <v>2024</v>
       </c>
       <c r="C8" s="29" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="D8" s="29" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="E8" s="69">
         <v>600</v>
@@ -12502,18 +12499,18 @@
         <v>33.333333333333336</v>
       </c>
       <c r="J8" s="24" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="71" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B9" s="74">
         <v>2022</v>
       </c>
       <c r="C9" s="65" t="s">
-        <v>421</v>
+        <v>410</v>
       </c>
       <c r="D9" s="65" t="s">
         <v>422</v>
@@ -12554,15 +12551,15 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="H12" s="42">
         <f>MEDIAN(H5:H9)</f>
-        <v>6.9050632911392409</v>
+        <v>7.6765708718947874</v>
       </c>
       <c r="I12" s="42">
-        <f>MEDIAN(I5,I7,I8,I9)</f>
-        <v>33.713541666666671</v>
+        <f>MEDIAN(I7,I8,I9)</f>
+        <v>33.333333333333336</v>
       </c>
       <c r="J12" t="s">
         <v>425</v>
@@ -12570,27 +12567,27 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="H13" s="42">
         <f>MIN(H5:H9)</f>
         <v>4.9249999999999998</v>
       </c>
       <c r="I13" s="42">
-        <f>MIN(I5,I7,I8,I9)</f>
+        <f>MIN(I7,I8,I9)</f>
         <v>23.64</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="H14" s="42">
         <f>MAX(H5:H9)</f>
         <v>10.017906336088155</v>
       </c>
       <c r="I14" s="42">
-        <f>MAX(I5,I7,I8,I9)</f>
+        <f>MAX(I7,I8,I9)</f>
         <v>79.55</v>
       </c>
     </row>
@@ -12693,13 +12690,16 @@
         <v>436</v>
       </c>
       <c r="E27" s="52">
-        <v>290</v>
+        <f>ROUND(E25,0)</f>
+        <v>289</v>
       </c>
       <c r="F27" s="52">
-        <v>410</v>
+        <f>ROUND(F25,0)</f>
+        <v>411</v>
       </c>
       <c r="G27" s="52">
-        <v>545</v>
+        <f>ROUND(G25,0)</f>
+        <v>547</v>
       </c>
       <c r="J27" s="28" t="s">
         <v>437</v>

</xml_diff>

<commit_message>
R7 (reliquat P0): Cover et marquages du workbook alignés sur la v2.1
Cover!A2: 'May 2026' -> 'Valuation as of 15-Jul-2026 (v2.1)'.
Cover!A41 (note 6 LBO): description v2 (4,0x, E3M+479bps ~7,16%, 1%
amort + sweep 75%, CIR single-count, rollover, exit 15x) + renvoi
explicite LBO_old = OBSOLETE.
Cover!A39 (note 4 comps): même classe de péremption, alignée sur les
comps du 15/07 (peers rafraîchis, EUR/USD 1,1424, fourchette formule).
LBO_full!A2: 'Build v2.1 · 15-Jul-2026 (...)' avec historique v1.0.
LBO_old: bannière OBSOLETE — DO NOT USE en rouge (A1/A2) + onglet
coloré rouge; aucune formule externe ne référence cette feuille
(vérifié). Recalc avec Excel UserName='Hamza Ben Chaouch' (pas de
régression lastModifiedBy). Checks 14/14, 0 erreur, moteur relançable
post-recalc (garde-fou muet). Commit 1 fichier exactement.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Sidetrade_Valuation_2026_v2.xlsx
+++ b/Sidetrade_Valuation_2026_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Abbah\Downloads\Portefolio\Portefolio\Sidetrade\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F051A0E-A785-4A38-944C-868FA7EBF77F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{166AB060-922B-46C8-B4D5-13E04260D50A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21840" tabRatio="500" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -48,10 +48,10 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="967" uniqueCount="776">
   <si>
-    <t>LBO AFFORDABILITY MODEL — BASE CASE  |  Max Entry EV for IRR targets</t>
-  </si>
-  <si>
-    <t>Simplified LBO: all unlevered FCF applied to debt service. Exit at fixed EBITDA multiple yr 5. IRR = equity return.</t>
+    <t>OBSOLETE — DO NOT USE · LBO AFFORDABILITY MODEL v1 (simplified) — superseded by LBO_full on 15-Jul-2026</t>
+  </si>
+  <si>
+    <t>OBSOLETE (kept for build history only — figures inconsistent with the current model). Simplified LBO: all unlevered FCF applied to debt service, exit at fixed EBITDA multiple yr 5, entry leverage 35% of EV.</t>
   </si>
   <si>
     <t>ASSUMPTIONS  (cross-linked from Inputs)</t>
@@ -192,7 +192,7 @@
     <t>SIDETRADE S.A. — VALUATION ANALYSIS</t>
   </si>
   <si>
-    <t>Order-to-Cash Intelligence Platform  |  Euronext Growth: ALBFR.PA  |  FY2025 base  |  May 2026</t>
+    <t>Order-to-Cash Intelligence Platform  |  Euronext Growth: ALBFR.PA  |  FY2025 base  |  Valuation as of 15-Jul-2026 (v2.1)</t>
   </si>
   <si>
     <t>CENTRAL VALUATION — STAND-ALONE BASIS</t>
@@ -327,13 +327,13 @@
     <t>3. Net debt: strict basis = gross financial debt €31.0m − cash+securities €16.3m = €14.7m. No adjustments for deferred revenue, earn-outs, or operating leases.</t>
   </si>
   <si>
-    <t>4. Trading comps: EV/Sales and EV/EBITDA on FY2026E estimates for BlackLine, BILL, nCino, Workiva. EUR-translated at 1.10 USD/EUR. Esker shown as reference (delisted).</t>
+    <t>4. Trading comps: EV/Sales forward (primary) and EV/non-GAAP operating income (proxy) on refreshed peers BlackLine, BILL, nCino, Workiva — prices as of 15-Jul-2026, May-2026 guidances, EUR/USD 1.1424. Selected range fully formula-driven from the peer table.</t>
   </si>
   <si>
     <t>5. Transaction comps: Esker, Coupa, Billtrust, Pagero, Bottomline. All include control premium (30-50%); not directly comparable to stand-alone DCF/trading EV.</t>
   </si>
   <si>
-    <t>6. LBO: simplified affordability model. All unlevered FCF applied to debt repayment. Exit at 15× EBITDA yr 5. Entry leverage 35%. IRR = equity return (MoM^(1/5)−1).</t>
+    <t>6. LBO: full affordability model (LBO_full tab, engine-solved via lbo_engine.py): entry leverage 4.0x EBITDA FY25, all-in E3M + 479bps ≈ 7.16%, 1% mandatory amortisation + 75% cash sweep, CIR single-count, founder rollover; exit at 15× EBITDA yr 5. The earlier simplified model (35% leverage, full sweep, all-FCF-to-debt) is kept in the LBO_old tab as OBSOLETE history — do not use.</t>
   </si>
   <si>
     <t>7. Margin path: point estimate = linear. Front-loaded and back-loaded paths computed in Margin_path tab. EV spread vs. linear: ±3-5%.</t>
@@ -1419,7 +1419,7 @@
     <t>SIDETRADE — LBO MODEL (FULL)</t>
   </si>
   <si>
-    <t>Build v1.0 · 10-Jun-2026 · per Build Spec v3 · Blue = input · Black = formula · Green = cross-sheet link</t>
+    <t>Build v2.1 · 15-Jul-2026 (CIR single-count fix, comps refresh 15/07, WACC bridge, Checks sheet) · originally v1.0 10-Jun-2026 per Build Spec v3 · Blue = input · Black = formula · Green = cross-sheet link</t>
   </si>
   <si>
     <t>Interest on OPENING debt (documented non-circular variant, Spec §3.4). Engine-solved values flagged in Source column.</t>
@@ -2394,7 +2394,7 @@
     <numFmt numFmtId="174" formatCode="0.00&quot;x&quot;"/>
     <numFmt numFmtId="175" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="46" x14ac:knownFonts="1">
+  <fonts count="48" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2682,6 +2682,18 @@
       <color rgb="FF808080"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FFC00000"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="10"/>
+      <color rgb="FFC00000"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
   <fills count="20">
     <fill>
@@ -2812,7 +2824,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="198">
+  <cellXfs count="200">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -3130,11 +3142,12 @@
     <xf numFmtId="166" fontId="42" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="42" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="45" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="46" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -3142,6 +3155,9 @@
     </xf>
     <xf numFmtId="0" fontId="13" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -3446,31 +3462,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="190" t="s">
+      <c r="A1" s="192" t="s">
         <v>47</v>
       </c>
-      <c r="B1" s="184"/>
-      <c r="C1" s="184"/>
-      <c r="D1" s="184"/>
-      <c r="E1" s="184"/>
+      <c r="B1" s="185"/>
+      <c r="C1" s="185"/>
+      <c r="D1" s="185"/>
+      <c r="E1" s="185"/>
     </row>
     <row r="2" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="189" t="s">
+      <c r="A2" s="191" t="s">
         <v>48</v>
       </c>
-      <c r="B2" s="184"/>
-      <c r="C2" s="184"/>
-      <c r="D2" s="184"/>
-      <c r="E2" s="184"/>
+      <c r="B2" s="185"/>
+      <c r="C2" s="185"/>
+      <c r="D2" s="185"/>
+      <c r="E2" s="185"/>
     </row>
     <row r="4" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="186" t="s">
+      <c r="A4" s="187" t="s">
         <v>49</v>
       </c>
-      <c r="B4" s="184"/>
-      <c r="C4" s="184"/>
-      <c r="D4" s="184"/>
-      <c r="E4" s="184"/>
+      <c r="B4" s="185"/>
+      <c r="C4" s="185"/>
+      <c r="D4" s="185"/>
+      <c r="E4" s="185"/>
     </row>
     <row r="5" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
@@ -3558,13 +3574,13 @@
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="186" t="s">
+      <c r="A11" s="187" t="s">
         <v>55</v>
       </c>
-      <c r="B11" s="184"/>
-      <c r="C11" s="184"/>
-      <c r="D11" s="184"/>
-      <c r="E11" s="184"/>
+      <c r="B11" s="185"/>
+      <c r="C11" s="185"/>
+      <c r="D11" s="185"/>
+      <c r="E11" s="185"/>
     </row>
     <row r="12" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
@@ -3579,13 +3595,13 @@
       </c>
     </row>
     <row r="14" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="186" t="s">
+      <c r="A14" s="187" t="s">
         <v>58</v>
       </c>
-      <c r="B14" s="184"/>
-      <c r="C14" s="184"/>
-      <c r="D14" s="184"/>
-      <c r="E14" s="184"/>
+      <c r="B14" s="185"/>
+      <c r="C14" s="185"/>
+      <c r="D14" s="185"/>
+      <c r="E14" s="185"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B15" s="15" t="s">
@@ -3682,13 +3698,13 @@
       </c>
     </row>
     <row r="21" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="186" t="s">
+      <c r="A21" s="187" t="s">
         <v>71</v>
       </c>
-      <c r="B21" s="184"/>
-      <c r="C21" s="184"/>
-      <c r="D21" s="184"/>
-      <c r="E21" s="184"/>
+      <c r="B21" s="185"/>
+      <c r="C21" s="185"/>
+      <c r="D21" s="185"/>
+      <c r="E21" s="185"/>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
@@ -3727,13 +3743,13 @@
       </c>
     </row>
     <row r="27" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="186" t="s">
+      <c r="A27" s="187" t="s">
         <v>76</v>
       </c>
-      <c r="B27" s="184"/>
-      <c r="C27" s="184"/>
-      <c r="D27" s="184"/>
-      <c r="E27" s="184"/>
+      <c r="B27" s="185"/>
+      <c r="C27" s="185"/>
+      <c r="D27" s="185"/>
+      <c r="E27" s="185"/>
     </row>
     <row r="28" spans="1:5" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="26" t="s">
@@ -3819,85 +3835,85 @@
       </c>
     </row>
     <row r="35" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="185" t="s">
+      <c r="A35" s="189" t="s">
         <v>89</v>
       </c>
-      <c r="B35" s="184"/>
-      <c r="C35" s="184"/>
-      <c r="D35" s="184"/>
-      <c r="E35" s="184"/>
+      <c r="B35" s="185"/>
+      <c r="C35" s="185"/>
+      <c r="D35" s="185"/>
+      <c r="E35" s="185"/>
     </row>
     <row r="36" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="188" t="s">
+      <c r="A36" s="190" t="s">
         <v>90</v>
       </c>
-      <c r="B36" s="184"/>
-      <c r="C36" s="184"/>
-      <c r="D36" s="184"/>
-      <c r="E36" s="184"/>
+      <c r="B36" s="185"/>
+      <c r="C36" s="185"/>
+      <c r="D36" s="185"/>
+      <c r="E36" s="185"/>
     </row>
     <row r="37" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="187" t="s">
+      <c r="A37" s="188" t="s">
         <v>91</v>
       </c>
-      <c r="B37" s="184"/>
-      <c r="C37" s="184"/>
-      <c r="D37" s="184"/>
-      <c r="E37" s="184"/>
+      <c r="B37" s="185"/>
+      <c r="C37" s="185"/>
+      <c r="D37" s="185"/>
+      <c r="E37" s="185"/>
     </row>
     <row r="38" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="188" t="s">
+      <c r="A38" s="190" t="s">
         <v>92</v>
       </c>
-      <c r="B38" s="184"/>
-      <c r="C38" s="184"/>
-      <c r="D38" s="184"/>
-      <c r="E38" s="184"/>
+      <c r="B38" s="185"/>
+      <c r="C38" s="185"/>
+      <c r="D38" s="185"/>
+      <c r="E38" s="185"/>
     </row>
     <row r="39" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="187" t="s">
+      <c r="A39" s="188" t="s">
         <v>93</v>
       </c>
-      <c r="B39" s="184"/>
-      <c r="C39" s="184"/>
-      <c r="D39" s="184"/>
-      <c r="E39" s="184"/>
+      <c r="B39" s="185"/>
+      <c r="C39" s="185"/>
+      <c r="D39" s="185"/>
+      <c r="E39" s="185"/>
     </row>
     <row r="40" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="188" t="s">
+      <c r="A40" s="190" t="s">
         <v>94</v>
       </c>
-      <c r="B40" s="184"/>
-      <c r="C40" s="184"/>
-      <c r="D40" s="184"/>
-      <c r="E40" s="184"/>
+      <c r="B40" s="185"/>
+      <c r="C40" s="185"/>
+      <c r="D40" s="185"/>
+      <c r="E40" s="185"/>
     </row>
     <row r="41" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="187" t="s">
+      <c r="A41" s="188" t="s">
         <v>95</v>
       </c>
-      <c r="B41" s="184"/>
-      <c r="C41" s="184"/>
-      <c r="D41" s="184"/>
-      <c r="E41" s="184"/>
+      <c r="B41" s="185"/>
+      <c r="C41" s="185"/>
+      <c r="D41" s="185"/>
+      <c r="E41" s="185"/>
     </row>
     <row r="42" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="188" t="s">
+      <c r="A42" s="190" t="s">
         <v>96</v>
       </c>
-      <c r="B42" s="184"/>
-      <c r="C42" s="184"/>
-      <c r="D42" s="184"/>
-      <c r="E42" s="184"/>
+      <c r="B42" s="185"/>
+      <c r="C42" s="185"/>
+      <c r="D42" s="185"/>
+      <c r="E42" s="185"/>
     </row>
     <row r="43" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="187" t="s">
+      <c r="A43" s="188" t="s">
         <v>97</v>
       </c>
-      <c r="B43" s="184"/>
-      <c r="C43" s="184"/>
-      <c r="D43" s="184"/>
-      <c r="E43" s="184"/>
+      <c r="B43" s="185"/>
+      <c r="C43" s="185"/>
+      <c r="D43" s="185"/>
+      <c r="E43" s="185"/>
     </row>
   </sheetData>
   <mergeCells count="16">
@@ -7781,15 +7797,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="191" t="s">
+      <c r="A1" s="193" t="s">
         <v>660</v>
       </c>
-      <c r="B1" s="184"/>
-      <c r="C1" s="184"/>
-      <c r="D1" s="184"/>
-      <c r="E1" s="184"/>
-      <c r="F1" s="184"/>
-      <c r="G1" s="184"/>
+      <c r="B1" s="185"/>
+      <c r="C1" s="185"/>
+      <c r="D1" s="185"/>
+      <c r="E1" s="185"/>
+      <c r="F1" s="185"/>
+      <c r="G1" s="185"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="14" t="s">
@@ -7938,15 +7954,15 @@
       <c r="G9" s="97"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="194" t="s">
+      <c r="A10" s="196" t="s">
         <v>674</v>
       </c>
-      <c r="B10" s="184"/>
-      <c r="C10" s="184"/>
-      <c r="D10" s="184"/>
-      <c r="E10" s="184"/>
-      <c r="F10" s="184"/>
-      <c r="G10" s="184"/>
+      <c r="B10" s="185"/>
+      <c r="C10" s="185"/>
+      <c r="D10" s="185"/>
+      <c r="E10" s="185"/>
+      <c r="F10" s="185"/>
+      <c r="G10" s="185"/>
     </row>
     <row r="11" spans="1:7" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
@@ -8093,13 +8109,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="191" t="s">
+      <c r="A1" s="193" t="s">
         <v>687</v>
       </c>
-      <c r="B1" s="184"/>
-      <c r="C1" s="184"/>
-      <c r="D1" s="184"/>
-      <c r="E1" s="184"/>
+      <c r="B1" s="185"/>
+      <c r="C1" s="185"/>
+      <c r="D1" s="185"/>
+      <c r="E1" s="185"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="14" t="s">
@@ -8121,12 +8137,12 @@
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="183" t="s">
+      <c r="A5" s="184" t="s">
         <v>689</v>
       </c>
-      <c r="B5" s="184"/>
-      <c r="C5" s="184"/>
-      <c r="D5" s="184"/>
+      <c r="B5" s="185"/>
+      <c r="C5" s="185"/>
+      <c r="D5" s="185"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
@@ -8146,12 +8162,12 @@
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="183" t="s">
+      <c r="A8" s="184" t="s">
         <v>690</v>
       </c>
-      <c r="B8" s="184"/>
-      <c r="C8" s="184"/>
-      <c r="D8" s="184"/>
+      <c r="B8" s="185"/>
+      <c r="C8" s="185"/>
+      <c r="D8" s="185"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
@@ -8234,12 +8250,12 @@
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="183" t="s">
+      <c r="A14" s="184" t="s">
         <v>696</v>
       </c>
-      <c r="B14" s="184"/>
-      <c r="C14" s="184"/>
-      <c r="D14" s="184"/>
+      <c r="B14" s="185"/>
+      <c r="C14" s="185"/>
+      <c r="D14" s="185"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
@@ -8259,12 +8275,12 @@
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="183" t="s">
+      <c r="A17" s="184" t="s">
         <v>698</v>
       </c>
-      <c r="B17" s="184"/>
-      <c r="C17" s="184"/>
-      <c r="D17" s="184"/>
+      <c r="B17" s="185"/>
+      <c r="C17" s="185"/>
+      <c r="D17" s="185"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="9" t="s">
@@ -8321,12 +8337,12 @@
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="183" t="s">
+      <c r="A22" s="184" t="s">
         <v>703</v>
       </c>
-      <c r="B22" s="184"/>
-      <c r="C22" s="184"/>
-      <c r="D22" s="184"/>
+      <c r="B22" s="185"/>
+      <c r="C22" s="185"/>
+      <c r="D22" s="185"/>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="9" t="s">
@@ -8359,13 +8375,13 @@
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" s="197" t="s">
+      <c r="A27" s="199" t="s">
         <v>708</v>
       </c>
-      <c r="B27" s="184"/>
-      <c r="C27" s="184"/>
-      <c r="D27" s="184"/>
-      <c r="E27" s="184"/>
+      <c r="B27" s="185"/>
+      <c r="C27" s="185"/>
+      <c r="D27" s="185"/>
+      <c r="E27" s="185"/>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="7" t="s">
@@ -8439,12 +8455,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="191" t="s">
+      <c r="A1" s="193" t="s">
         <v>714</v>
       </c>
-      <c r="B1" s="184"/>
-      <c r="C1" s="184"/>
-      <c r="D1" s="184"/>
+      <c r="B1" s="185"/>
+      <c r="C1" s="185"/>
+      <c r="D1" s="185"/>
     </row>
     <row r="3" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
@@ -8879,13 +8895,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="191" t="s">
+      <c r="A1" s="193" t="s">
         <v>98</v>
       </c>
-      <c r="B1" s="184"/>
-      <c r="C1" s="184"/>
-      <c r="D1" s="184"/>
-      <c r="E1" s="184"/>
+      <c r="B1" s="185"/>
+      <c r="C1" s="185"/>
+      <c r="D1" s="185"/>
+      <c r="E1" s="185"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="14" t="s">
@@ -8910,13 +8926,13 @@
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="183" t="s">
+      <c r="A5" s="184" t="s">
         <v>105</v>
       </c>
-      <c r="B5" s="184"/>
-      <c r="C5" s="184"/>
-      <c r="D5" s="184"/>
-      <c r="E5" s="184"/>
+      <c r="B5" s="185"/>
+      <c r="C5" s="185"/>
+      <c r="D5" s="185"/>
+      <c r="E5" s="185"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
@@ -9024,13 +9040,13 @@
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="183" t="s">
+      <c r="A13" s="184" t="s">
         <v>118</v>
       </c>
-      <c r="B13" s="184"/>
-      <c r="C13" s="184"/>
-      <c r="D13" s="184"/>
-      <c r="E13" s="184"/>
+      <c r="B13" s="185"/>
+      <c r="C13" s="185"/>
+      <c r="D13" s="185"/>
+      <c r="E13" s="185"/>
     </row>
     <row r="14" spans="1:5" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
@@ -9112,13 +9128,13 @@
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="183" t="s">
+      <c r="A20" s="184" t="s">
         <v>127</v>
       </c>
-      <c r="B20" s="184"/>
-      <c r="C20" s="184"/>
-      <c r="D20" s="184"/>
-      <c r="E20" s="184"/>
+      <c r="B20" s="185"/>
+      <c r="C20" s="185"/>
+      <c r="D20" s="185"/>
+      <c r="E20" s="185"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="9" t="s">
@@ -9246,13 +9262,13 @@
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A29" s="183" t="s">
+      <c r="A29" s="184" t="s">
         <v>138</v>
       </c>
-      <c r="B29" s="184"/>
-      <c r="C29" s="184"/>
-      <c r="D29" s="184"/>
-      <c r="E29" s="184"/>
+      <c r="B29" s="185"/>
+      <c r="C29" s="185"/>
+      <c r="D29" s="185"/>
+      <c r="E29" s="185"/>
     </row>
     <row r="30" spans="1:5" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="9" t="s">
@@ -9340,13 +9356,13 @@
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A36" s="183" t="s">
+      <c r="A36" s="184" t="s">
         <v>149</v>
       </c>
-      <c r="B36" s="184"/>
-      <c r="C36" s="184"/>
-      <c r="D36" s="184"/>
-      <c r="E36" s="184"/>
+      <c r="B36" s="185"/>
+      <c r="C36" s="185"/>
+      <c r="D36" s="185"/>
+      <c r="E36" s="185"/>
     </row>
     <row r="37" spans="1:5" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="9" t="s">
@@ -9400,13 +9416,13 @@
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A41" s="183" t="s">
+      <c r="A41" s="184" t="s">
         <v>156</v>
       </c>
-      <c r="B41" s="184"/>
-      <c r="C41" s="184"/>
-      <c r="D41" s="184"/>
-      <c r="E41" s="184"/>
+      <c r="B41" s="185"/>
+      <c r="C41" s="185"/>
+      <c r="D41" s="185"/>
+      <c r="E41" s="185"/>
     </row>
     <row r="42" spans="1:5" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="9" t="s">
@@ -9600,18 +9616,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="185" t="s">
+      <c r="A1" s="189" t="s">
         <v>180</v>
       </c>
-      <c r="B1" s="184"/>
-      <c r="C1" s="184"/>
-      <c r="D1" s="184"/>
+      <c r="B1" s="185"/>
+      <c r="C1" s="185"/>
+      <c r="D1" s="185"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="183" t="s">
+      <c r="A3" s="184" t="s">
         <v>181</v>
       </c>
-      <c r="B3" s="184"/>
+      <c r="B3" s="185"/>
       <c r="C3" s="3" t="s">
         <v>182</v>
       </c>
@@ -9819,10 +9835,10 @@
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="183" t="s">
+      <c r="A19" s="184" t="s">
         <v>209</v>
       </c>
-      <c r="B19" s="184"/>
+      <c r="B19" s="185"/>
       <c r="C19" s="3" t="s">
         <v>182</v>
       </c>
@@ -9904,10 +9920,10 @@
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="183" t="s">
+      <c r="A26" s="184" t="s">
         <v>219</v>
       </c>
-      <c r="B26" s="184"/>
+      <c r="B26" s="185"/>
       <c r="C26" s="3" t="s">
         <v>220</v>
       </c>
@@ -9992,10 +10008,10 @@
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="183" t="s">
+      <c r="A35" s="184" t="s">
         <v>233</v>
       </c>
-      <c r="B35" s="184"/>
+      <c r="B35" s="185"/>
       <c r="C35" s="3" t="s">
         <v>234</v>
       </c>
@@ -10098,10 +10114,10 @@
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="183" t="s">
+      <c r="A45" s="184" t="s">
         <v>246</v>
       </c>
-      <c r="B45" s="184"/>
+      <c r="B45" s="185"/>
       <c r="C45" s="3" t="s">
         <v>247</v>
       </c>
@@ -10150,10 +10166,10 @@
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="183" t="s">
+      <c r="A51" s="184" t="s">
         <v>254</v>
       </c>
-      <c r="B51" s="184"/>
+      <c r="B51" s="185"/>
       <c r="C51" s="3" t="s">
         <v>247</v>
       </c>
@@ -10215,10 +10231,10 @@
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A58" s="183" t="s">
+      <c r="A58" s="184" t="s">
         <v>264</v>
       </c>
-      <c r="B58" s="184"/>
+      <c r="B58" s="185"/>
       <c r="C58" s="3" t="s">
         <v>247</v>
       </c>
@@ -10295,10 +10311,10 @@
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A67" s="183" t="s">
+      <c r="A67" s="184" t="s">
         <v>274</v>
       </c>
-      <c r="B67" s="184"/>
+      <c r="B67" s="185"/>
     </row>
     <row r="68" spans="1:4" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="9" t="s">
@@ -10350,27 +10366,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="191" t="s">
+      <c r="A1" s="193" t="s">
         <v>279</v>
       </c>
-      <c r="B1" s="184"/>
-      <c r="C1" s="184"/>
-      <c r="D1" s="184"/>
-      <c r="E1" s="184"/>
-      <c r="F1" s="184"/>
-      <c r="G1" s="184"/>
-      <c r="H1" s="184"/>
-      <c r="I1" s="184"/>
-      <c r="J1" s="184"/>
-      <c r="K1" s="184"/>
-      <c r="L1" s="184"/>
-      <c r="M1" s="184"/>
-      <c r="N1" s="184"/>
-      <c r="O1" s="184"/>
-      <c r="P1" s="184"/>
-      <c r="Q1" s="184"/>
-      <c r="R1" s="184"/>
-      <c r="S1" s="184"/>
+      <c r="B1" s="185"/>
+      <c r="C1" s="185"/>
+      <c r="D1" s="185"/>
+      <c r="E1" s="185"/>
+      <c r="F1" s="185"/>
+      <c r="G1" s="185"/>
+      <c r="H1" s="185"/>
+      <c r="I1" s="185"/>
+      <c r="J1" s="185"/>
+      <c r="K1" s="185"/>
+      <c r="L1" s="185"/>
+      <c r="M1" s="185"/>
+      <c r="N1" s="185"/>
+      <c r="O1" s="185"/>
+      <c r="P1" s="185"/>
+      <c r="Q1" s="185"/>
+      <c r="R1" s="185"/>
+      <c r="S1" s="185"/>
     </row>
     <row r="2" spans="1:19" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="54" t="s">
@@ -10378,36 +10394,36 @@
       </c>
     </row>
     <row r="3" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="192" t="s">
+      <c r="B3" s="194" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="184"/>
-      <c r="D3" s="184"/>
-      <c r="E3" s="192" t="s">
+      <c r="C3" s="185"/>
+      <c r="D3" s="185"/>
+      <c r="E3" s="194" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="184"/>
-      <c r="G3" s="184"/>
-      <c r="H3" s="192" t="s">
+      <c r="F3" s="185"/>
+      <c r="G3" s="185"/>
+      <c r="H3" s="194" t="s">
         <v>11</v>
       </c>
-      <c r="I3" s="184"/>
-      <c r="J3" s="184"/>
-      <c r="K3" s="192" t="s">
+      <c r="I3" s="185"/>
+      <c r="J3" s="185"/>
+      <c r="K3" s="194" t="s">
         <v>12</v>
       </c>
-      <c r="L3" s="184"/>
-      <c r="M3" s="184"/>
-      <c r="N3" s="192" t="s">
+      <c r="L3" s="185"/>
+      <c r="M3" s="185"/>
+      <c r="N3" s="194" t="s">
         <v>13</v>
       </c>
-      <c r="O3" s="184"/>
-      <c r="P3" s="184"/>
-      <c r="Q3" s="193" t="s">
+      <c r="O3" s="185"/>
+      <c r="P3" s="185"/>
+      <c r="Q3" s="195" t="s">
         <v>281</v>
       </c>
-      <c r="R3" s="184"/>
-      <c r="S3" s="184"/>
+      <c r="R3" s="185"/>
+      <c r="S3" s="185"/>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B4" s="55" t="s">
@@ -11688,16 +11704,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="185" t="s">
+      <c r="A1" s="189" t="s">
         <v>317</v>
       </c>
-      <c r="B1" s="184"/>
-      <c r="C1" s="184"/>
-      <c r="D1" s="184"/>
-      <c r="E1" s="184"/>
-      <c r="F1" s="184"/>
-      <c r="G1" s="184"/>
-      <c r="H1" s="184"/>
+      <c r="B1" s="185"/>
+      <c r="C1" s="185"/>
+      <c r="D1" s="185"/>
+      <c r="E1" s="185"/>
+      <c r="F1" s="185"/>
+      <c r="G1" s="185"/>
+      <c r="H1" s="185"/>
     </row>
     <row r="2" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="14" t="s">
@@ -11705,15 +11721,15 @@
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="194" t="s">
+      <c r="A4" s="196" t="s">
         <v>319</v>
       </c>
-      <c r="B4" s="184"/>
-      <c r="C4" s="184"/>
-      <c r="D4" s="184"/>
-      <c r="E4" s="184"/>
-      <c r="F4" s="184"/>
-      <c r="G4" s="184"/>
+      <c r="B4" s="185"/>
+      <c r="C4" s="185"/>
+      <c r="D4" s="185"/>
+      <c r="E4" s="185"/>
+      <c r="F4" s="185"/>
+      <c r="G4" s="185"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
@@ -11866,15 +11882,15 @@
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="194" t="s">
+      <c r="A14" s="196" t="s">
         <v>322</v>
       </c>
-      <c r="B14" s="184"/>
-      <c r="C14" s="184"/>
-      <c r="D14" s="184"/>
-      <c r="E14" s="184"/>
-      <c r="F14" s="184"/>
-      <c r="G14" s="184"/>
+      <c r="B14" s="185"/>
+      <c r="C14" s="185"/>
+      <c r="D14" s="185"/>
+      <c r="E14" s="185"/>
+      <c r="F14" s="185"/>
+      <c r="G14" s="185"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
@@ -12053,13 +12069,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="185" t="s">
+      <c r="A1" s="189" t="s">
         <v>326</v>
       </c>
-      <c r="B1" s="184"/>
-      <c r="C1" s="184"/>
-      <c r="D1" s="184"/>
-      <c r="E1" s="184"/>
+      <c r="B1" s="185"/>
+      <c r="C1" s="185"/>
+      <c r="D1" s="185"/>
+      <c r="E1" s="185"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="14" t="s">
@@ -12115,13 +12131,13 @@
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="194" t="s">
+      <c r="A8" s="196" t="s">
         <v>332</v>
       </c>
-      <c r="B8" s="184"/>
-      <c r="C8" s="184"/>
-      <c r="D8" s="184"/>
-      <c r="E8" s="184"/>
+      <c r="B8" s="185"/>
+      <c r="C8" s="185"/>
+      <c r="D8" s="185"/>
+      <c r="E8" s="185"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
@@ -12224,13 +12240,13 @@
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="194" t="s">
+      <c r="A15" s="196" t="s">
         <v>338</v>
       </c>
-      <c r="B15" s="184"/>
-      <c r="C15" s="184"/>
-      <c r="D15" s="184"/>
-      <c r="E15" s="184"/>
+      <c r="B15" s="185"/>
+      <c r="C15" s="185"/>
+      <c r="D15" s="185"/>
+      <c r="E15" s="185"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
@@ -12418,13 +12434,13 @@
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" s="194" t="s">
+      <c r="A27" s="196" t="s">
         <v>354</v>
       </c>
-      <c r="B27" s="184"/>
-      <c r="C27" s="184"/>
-      <c r="D27" s="184"/>
-      <c r="E27" s="184"/>
+      <c r="B27" s="185"/>
+      <c r="C27" s="185"/>
+      <c r="D27" s="185"/>
+      <c r="E27" s="185"/>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="9" t="s">
@@ -12629,17 +12645,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="195" t="s">
+      <c r="A1" s="197" t="s">
         <v>366</v>
       </c>
-      <c r="B1" s="184"/>
-      <c r="C1" s="184"/>
-      <c r="D1" s="184"/>
-      <c r="E1" s="184"/>
-      <c r="F1" s="184"/>
-      <c r="G1" s="184"/>
-      <c r="H1" s="184"/>
-      <c r="I1" s="184"/>
+      <c r="B1" s="185"/>
+      <c r="C1" s="185"/>
+      <c r="D1" s="185"/>
+      <c r="E1" s="185"/>
+      <c r="F1" s="185"/>
+      <c r="G1" s="185"/>
+      <c r="H1" s="185"/>
+      <c r="I1" s="185"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="155" t="s">
@@ -12824,17 +12840,17 @@
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="196" t="s">
+      <c r="A11" s="198" t="s">
         <v>392</v>
       </c>
-      <c r="B11" s="184"/>
-      <c r="C11" s="184"/>
-      <c r="D11" s="184"/>
-      <c r="E11" s="184"/>
-      <c r="F11" s="184"/>
-      <c r="G11" s="184"/>
-      <c r="H11" s="184"/>
-      <c r="I11" s="184"/>
+      <c r="B11" s="185"/>
+      <c r="C11" s="185"/>
+      <c r="D11" s="185"/>
+      <c r="E11" s="185"/>
+      <c r="F11" s="185"/>
+      <c r="G11" s="185"/>
+      <c r="H11" s="185"/>
+      <c r="I11" s="185"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="171" t="s">
@@ -12876,17 +12892,17 @@
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" s="196" t="s">
+      <c r="A16" s="198" t="s">
         <v>396</v>
       </c>
-      <c r="B16" s="184"/>
-      <c r="C16" s="184"/>
-      <c r="D16" s="184"/>
-      <c r="E16" s="184"/>
-      <c r="F16" s="184"/>
-      <c r="G16" s="184"/>
-      <c r="H16" s="184"/>
-      <c r="I16" s="184"/>
+      <c r="B16" s="185"/>
+      <c r="C16" s="185"/>
+      <c r="D16" s="185"/>
+      <c r="E16" s="185"/>
+      <c r="F16" s="185"/>
+      <c r="G16" s="185"/>
+      <c r="H16" s="185"/>
+      <c r="I16" s="185"/>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="171" t="s">
@@ -13038,18 +13054,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="185" t="s">
+      <c r="A1" s="189" t="s">
         <v>410</v>
       </c>
-      <c r="B1" s="184"/>
-      <c r="C1" s="184"/>
-      <c r="D1" s="184"/>
-      <c r="E1" s="184"/>
-      <c r="F1" s="184"/>
-      <c r="G1" s="184"/>
-      <c r="H1" s="184"/>
-      <c r="I1" s="184"/>
-      <c r="J1" s="184"/>
+      <c r="B1" s="185"/>
+      <c r="C1" s="185"/>
+      <c r="D1" s="185"/>
+      <c r="E1" s="185"/>
+      <c r="F1" s="185"/>
+      <c r="G1" s="185"/>
+      <c r="H1" s="185"/>
+      <c r="I1" s="185"/>
+      <c r="J1" s="185"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="73" t="s">
@@ -13256,17 +13272,17 @@
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A11" s="194" t="s">
+      <c r="A11" s="196" t="s">
         <v>440</v>
       </c>
-      <c r="B11" s="184"/>
-      <c r="C11" s="184"/>
-      <c r="D11" s="184"/>
-      <c r="E11" s="184"/>
-      <c r="F11" s="184"/>
-      <c r="G11" s="184"/>
-      <c r="H11" s="184"/>
-      <c r="I11" s="184"/>
+      <c r="B11" s="185"/>
+      <c r="C11" s="185"/>
+      <c r="D11" s="185"/>
+      <c r="E11" s="185"/>
+      <c r="F11" s="185"/>
+      <c r="G11" s="185"/>
+      <c r="H11" s="185"/>
+      <c r="I11" s="185"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
@@ -13311,18 +13327,18 @@
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A16" s="194" t="s">
+      <c r="A16" s="196" t="s">
         <v>443</v>
       </c>
-      <c r="B16" s="184"/>
-      <c r="C16" s="184"/>
-      <c r="D16" s="184"/>
-      <c r="E16" s="184"/>
-      <c r="F16" s="184"/>
-      <c r="G16" s="184"/>
-      <c r="H16" s="184"/>
-      <c r="I16" s="184"/>
-      <c r="J16" s="184"/>
+      <c r="B16" s="185"/>
+      <c r="C16" s="185"/>
+      <c r="D16" s="185"/>
+      <c r="E16" s="185"/>
+      <c r="F16" s="185"/>
+      <c r="G16" s="185"/>
+      <c r="H16" s="185"/>
+      <c r="I16" s="185"/>
+      <c r="J16" s="185"/>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="76" t="s">
@@ -13442,6 +13458,9 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+  <sheetPr>
+    <tabColor rgb="FFC00000"/>
+  </sheetPr>
   <dimension ref="A1:I35"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -13452,28 +13471,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="185" t="s">
+      <c r="A1" s="186" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="184"/>
-      <c r="C1" s="184"/>
-      <c r="D1" s="184"/>
-      <c r="E1" s="184"/>
-      <c r="F1" s="184"/>
-      <c r="G1" s="184"/>
-      <c r="H1" s="184"/>
-      <c r="I1" s="184"/>
+      <c r="B1" s="185"/>
+      <c r="C1" s="185"/>
+      <c r="D1" s="185"/>
+      <c r="E1" s="185"/>
+      <c r="F1" s="185"/>
+      <c r="G1" s="185"/>
+      <c r="H1" s="185"/>
+      <c r="I1" s="185"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="183" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="183" t="s">
+      <c r="A4" s="184" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="184"/>
+      <c r="B4" s="185"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
@@ -13514,10 +13533,10 @@
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="183" t="s">
+      <c r="A10" s="184" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="184"/>
+      <c r="B10" s="185"/>
       <c r="C10" s="3" t="s">
         <v>9</v>
       </c>
@@ -13650,10 +13669,10 @@
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" s="183" t="s">
+      <c r="A16" s="184" t="s">
         <v>19</v>
       </c>
-      <c r="B16" s="184"/>
+      <c r="B16" s="185"/>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
@@ -13783,10 +13802,10 @@
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A26" s="183" t="s">
+      <c r="A26" s="184" t="s">
         <v>36</v>
       </c>
-      <c r="B26" s="184"/>
+      <c r="B26" s="185"/>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="9" t="s">

</xml_diff>